<commit_message>
Small spec updates/fixes + addition of docs/Evolute-Simultaneous_Charging.pdf.
</commit_message>
<xml_diff>
--- a/docs/Rough_kW_kVA_Table.xlsx
+++ b/docs/Rough_kW_kVA_Table.xlsx
@@ -10,6 +10,15 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" name="BREAKER_RATING_A" vbProcedure="false">Sheet1!$B$14</definedName>
+    <definedName function="false" hidden="false" name="CONTINUOUS_DUTY_DERATE" vbProcedure="false">Sheet1!$B$15</definedName>
+    <definedName function="false" hidden="false" name="ev_apparent_power_kva" vbProcedure="false">Sheet1!$B$18</definedName>
+    <definedName function="false" hidden="false" name="ev_pilot_current_a" vbProcedure="false">Sheet1!$B$17</definedName>
+    <definedName function="false" hidden="false" name="ev_real_power_kw" vbProcedure="false">Sheet1!$B$19</definedName>
+    <definedName function="false" hidden="false" name="EV_TRUE_POWER_FACTOR" vbProcedure="false">Sheet1!$B$16</definedName>
+    <definedName function="false" hidden="false" name="PANEL_VOLTAGE_V" vbProcedure="false">Sheet1!$B$13</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -20,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t xml:space="preserve">kW</t>
   </si>
@@ -29,6 +38,27 @@
   </si>
   <si>
     <t xml:space="preserve">PF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PANEL_VOLTAGE_V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BREAKER_RATING_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONTINUOUS_DUTY_DERATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV_TRUE_POWER_FACTOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ev_pilot_current_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ev_apparent_power_kva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ev_real_power_kw</t>
   </si>
 </sst>
 </file>
@@ -44,6 +74,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -103,12 +134,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -129,9 +164,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.39"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="11.52"/>
   </cols>
   <sheetData>
@@ -144,13 +180,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="2" t="n">
         <v>6.666</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="n">
@@ -163,13 +199,14 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="2" t="n">
+        <f aca="false">B16</f>
         <v>0.99</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="1" t="n">
@@ -182,7 +219,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="1" t="n">
@@ -195,7 +232,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="1" t="n">
@@ -208,7 +245,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="1" t="n">
@@ -221,7 +258,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="2" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="n">
@@ -234,7 +271,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="1" t="n">
@@ -247,7 +284,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="2" t="n">
         <v>8</v>
       </c>
       <c r="D9" s="1" t="n">
@@ -260,7 +297,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="D10" s="1" t="n">
@@ -273,7 +310,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="0" t="n">
+      <c r="C11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="1" t="n">
@@ -283,6 +320,65 @@
       <c r="E11" s="1" t="n">
         <f aca="false">D11/$B$3</f>
         <v>67.3333333333333</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <f aca="false"> BREAKER_RATING_A * CONTINUOUS_DUTY_DERATE</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <f aca="false"> PANEL_VOLTAGE_V * ev_pilot_current_a / 1000</f>
+        <v>6.656</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="0" t="n">
+        <f aca="false"> ev_apparent_power_kva * EV_TRUE_POWER_FACTOR</f>
+        <v>6.58944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>